<commit_message>
fix single entry edit
</commit_message>
<xml_diff>
--- a/data/horizon_cadence_transformed.xlsx
+++ b/data/horizon_cadence_transformed.xlsx
@@ -1143,7 +1143,7 @@
         </is>
       </c>
       <c r="C16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
@@ -1158,12 +1158,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Automation</t>
+          <t>automation</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Explore</t>
+          <t>explore</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1173,7 +1173,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>automation,bedag,oiz,swisscom</t>
+          <t>automation, bedag, oiz, swisscom</t>
         </is>
       </c>
       <c r="K16" t="inlineStr"/>

</xml_diff>